<commit_message>
implmenentacion de creacion de hoja de vida y descargar excel y pdf
</commit_message>
<xml_diff>
--- a/storage/app/templates/plantilla_hoja_vida_equipos.xlsx
+++ b/storage/app/templates/plantilla_hoja_vida_equipos.xlsx
@@ -424,11 +424,11 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -436,19 +436,19 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -456,7 +456,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -468,11 +468,11 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -552,15 +552,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>154440</xdr:colOff>
+      <xdr:colOff>102600</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>117720</xdr:rowOff>
+      <xdr:rowOff>146160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>603000</xdr:colOff>
+      <xdr:colOff>321840</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>322200</xdr:rowOff>
+      <xdr:rowOff>349200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -573,8 +573,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="428760" y="280440"/>
-          <a:ext cx="2301480" cy="774000"/>
+          <a:off x="376920" y="308880"/>
+          <a:ext cx="1814400" cy="772560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -770,20 +770,22 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="10.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="6.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="6.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="2.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="15.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="12.12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -938,13 +940,17 @@
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2"/>
-      <c r="B9" s="10"/>
+      <c r="B9" s="10" t="s">
+        <v>11</v>
+      </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
       <c r="G9" s="10"/>
-      <c r="H9" s="11"/>
+      <c r="H9" s="11" t="s">
+        <v>12</v>
+      </c>
       <c r="I9" s="11"/>
       <c r="J9" s="11"/>
       <c r="K9" s="12"/>
@@ -955,7 +961,7 @@
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2"/>
       <c r="B10" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
@@ -963,7 +969,7 @@
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
       <c r="H10" s="11" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I10" s="11"/>
       <c r="J10" s="11"/>
@@ -975,7 +981,7 @@
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2"/>
       <c r="B11" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
@@ -983,7 +989,7 @@
       <c r="F11" s="10"/>
       <c r="G11" s="10"/>
       <c r="H11" s="11" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I11" s="11"/>
       <c r="J11" s="11"/>
@@ -994,205 +1000,201 @@
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
-      <c r="B12" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
+      <c r="B12" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="I12" s="14"/>
+      <c r="J12" s="14"/>
       <c r="K12" s="12"/>
       <c r="L12" s="12"/>
       <c r="M12" s="12"/>
       <c r="N12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2"/>
-      <c r="B13" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="I13" s="14"/>
-      <c r="J13" s="14"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="12"/>
+      <c r="B13" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
       <c r="N13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
-      <c r="B14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9"/>
+      <c r="B14" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="L14" s="15"/>
+      <c r="M14" s="15"/>
       <c r="N14" s="2"/>
     </row>
-    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2"/>
       <c r="B15" s="10" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
-      <c r="E15" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
+      <c r="E15" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
       <c r="H15" s="11" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="I15" s="11"/>
       <c r="J15" s="11"/>
-      <c r="K15" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
+      <c r="K15" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="L15" s="15"/>
+      <c r="M15" s="15"/>
       <c r="N15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
       <c r="B16" s="10" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
       <c r="E16" s="11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F16" s="11"/>
       <c r="G16" s="11"/>
       <c r="H16" s="11" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I16" s="11"/>
       <c r="J16" s="11"/>
-      <c r="K16" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
+      <c r="K16" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="L16" s="15"/>
+      <c r="M16" s="15"/>
       <c r="N16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2"/>
-      <c r="B17" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
+      <c r="B17" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="I17" s="14"/>
+      <c r="J17" s="14"/>
       <c r="K17" s="16" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="L17" s="16"/>
       <c r="M17" s="16"/>
       <c r="N17" s="2"/>
     </row>
-    <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2"/>
-      <c r="B18" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="L18" s="12"/>
-      <c r="M18" s="12"/>
+      <c r="B18" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
       <c r="N18" s="2"/>
     </row>
-    <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2"/>
-      <c r="B19" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="9"/>
-      <c r="M19" s="9"/>
+      <c r="B19" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="17"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F19" s="19"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="I19" s="19"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="L19" s="19"/>
+      <c r="M19" s="20"/>
       <c r="N19" s="2"/>
     </row>
-    <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2"/>
-      <c r="B20" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="F20" s="19"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="I20" s="19"/>
-      <c r="J20" s="18"/>
-      <c r="K20" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="L20" s="19"/>
-      <c r="M20" s="20"/>
+      <c r="B20" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="21"/>
+      <c r="L20" s="21"/>
+      <c r="M20" s="21"/>
       <c r="N20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2"/>
-      <c r="B21" s="21" t="s">
-        <v>41</v>
-      </c>
+      <c r="B21" s="21"/>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
@@ -1208,7 +1210,9 @@
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2"/>
-      <c r="B22" s="21"/>
+      <c r="B22" s="21" t="s">
+        <v>42</v>
+      </c>
       <c r="C22" s="21"/>
       <c r="D22" s="21"/>
       <c r="E22" s="21"/>
@@ -1224,9 +1228,7 @@
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="2"/>
-      <c r="B23" s="21" t="s">
-        <v>42</v>
-      </c>
+      <c r="B23" s="21"/>
       <c r="C23" s="21"/>
       <c r="D23" s="21"/>
       <c r="E23" s="21"/>
@@ -1242,7 +1244,9 @@
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2"/>
-      <c r="B24" s="21"/>
+      <c r="B24" s="21" t="s">
+        <v>43</v>
+      </c>
       <c r="C24" s="21"/>
       <c r="D24" s="21"/>
       <c r="E24" s="21"/>
@@ -1258,9 +1262,7 @@
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2"/>
-      <c r="B25" s="21" t="s">
-        <v>43</v>
-      </c>
+      <c r="B25" s="21"/>
       <c r="C25" s="21"/>
       <c r="D25" s="21"/>
       <c r="E25" s="21"/>
@@ -1276,25 +1278,25 @@
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2"/>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
-      <c r="I26" s="21"/>
-      <c r="J26" s="21"/>
-      <c r="K26" s="21"/>
-      <c r="L26" s="21"/>
-      <c r="M26" s="21"/>
+      <c r="B26" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="22"/>
+      <c r="J26" s="22"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="22"/>
+      <c r="M26" s="22"/>
       <c r="N26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="2"/>
-      <c r="B27" s="22" t="s">
-        <v>44</v>
-      </c>
+      <c r="B27" s="22"/>
       <c r="C27" s="22"/>
       <c r="D27" s="22"/>
       <c r="E27" s="22"/>
@@ -1308,9 +1310,11 @@
       <c r="M27" s="22"/>
       <c r="N27" s="2"/>
     </row>
-    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2"/>
-      <c r="B28" s="22"/>
+      <c r="B28" s="22" t="s">
+        <v>45</v>
+      </c>
       <c r="C28" s="22"/>
       <c r="D28" s="22"/>
       <c r="E28" s="22"/>
@@ -1324,11 +1328,9 @@
       <c r="M28" s="22"/>
       <c r="N28" s="2"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="29.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="2"/>
-      <c r="B29" s="22" t="s">
-        <v>45</v>
-      </c>
+      <c r="B29" s="22"/>
       <c r="C29" s="22"/>
       <c r="D29" s="22"/>
       <c r="E29" s="22"/>
@@ -1342,38 +1344,23 @@
       <c r="M29" s="22"/>
       <c r="N29" s="2"/>
     </row>
-    <row r="30" customFormat="false" ht="29.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2"/>
-      <c r="B30" s="22"/>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="22"/>
-      <c r="H30" s="22"/>
-      <c r="I30" s="22"/>
-      <c r="J30" s="22"/>
-      <c r="K30" s="22"/>
-      <c r="L30" s="22"/>
-      <c r="M30" s="22"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
+      <c r="L30" s="2"/>
+      <c r="M30" s="2"/>
       <c r="N30" s="2"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
-      <c r="N31" s="2"/>
-    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="48">
     <mergeCell ref="B2:D4"/>
@@ -1385,19 +1372,23 @@
     <mergeCell ref="B5:M5"/>
     <mergeCell ref="B6:G6"/>
     <mergeCell ref="H6:J6"/>
-    <mergeCell ref="K6:M13"/>
+    <mergeCell ref="K6:M12"/>
     <mergeCell ref="B7:J7"/>
-    <mergeCell ref="B8:G9"/>
-    <mergeCell ref="H8:J9"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="H9:J9"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="H10:J10"/>
     <mergeCell ref="B11:G11"/>
     <mergeCell ref="H11:J11"/>
     <mergeCell ref="B12:G12"/>
     <mergeCell ref="H12:J12"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="B14:M14"/>
+    <mergeCell ref="B13:M13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="K14:M14"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:J15"/>
@@ -1410,24 +1401,20 @@
     <mergeCell ref="E17:G17"/>
     <mergeCell ref="H17:J17"/>
     <mergeCell ref="K17:M17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:J18"/>
-    <mergeCell ref="K18:M18"/>
-    <mergeCell ref="B19:M19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="B21:M22"/>
-    <mergeCell ref="B23:M24"/>
-    <mergeCell ref="B25:M26"/>
-    <mergeCell ref="B27:M28"/>
-    <mergeCell ref="B29:M30"/>
+    <mergeCell ref="B18:M18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="B20:M21"/>
+    <mergeCell ref="B22:M23"/>
+    <mergeCell ref="B24:M25"/>
+    <mergeCell ref="B26:M27"/>
+    <mergeCell ref="B28:M29"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="65" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>